<commit_message>
refactor pour séparation UI / métier
</commit_message>
<xml_diff>
--- a/PartList_PCB_A_B_v2.xlsx
+++ b/PartList_PCB_A_B_v2.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -458,10 +458,14 @@
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="29" customWidth="1" min="6" max="6"/>
     <col width="31" customWidth="1" min="7" max="7"/>
-    <col width="70" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
     <col width="5" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="70" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="33" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="59" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -520,6 +524,26 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Assemble_JLC</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>JLC_Type</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>LCSC_Status</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>JLC_Notes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -575,6 +599,26 @@
           <t>Conforme au setup actuel: board nodemcu-32s. DevKit achete assemble.</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Module externe (DevKit complet)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -630,6 +674,26 @@
           <t>Verifier entraxe exact du modele DevKit retenu.</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Connecteur mecanique, option selon strategie assemblage</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -685,6 +749,26 @@
           <t>VIN cible 12V, marge recommandee jusqu a 24V.</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>THT/Manual</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Completer un code LCSC (Cxxxx) pour PCBA auto.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -740,6 +824,26 @@
           <t>Alimente pin 5V du DevKit et peripheriques 5V.</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Module buck pre-assemble ou design discret a figer</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -795,6 +899,26 @@
           <t>Dimensionner selon courant max et tension transitoire.</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>SMT+THT mix</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Completer un code LCSC (Cxxxx) pour PCBA auto.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -850,6 +974,26 @@
           <t>Utilise par firmware via hd44780_I2Cexp.</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Module LCD + backpack souvent hors catalogue SMT standard</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -874,7 +1018,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -905,6 +1049,26 @@
           <t>Adresses firmware: 0x48..0x4B.</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>SMT</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Completer un code LCSC (Cxxxx) ou choisir capteur dispo JLC.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -960,6 +1124,26 @@
           <t>Adresses firmware: 0x23/0x5C.</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>SMT</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Completer un code LCSC (Cxxxx) pour PCBA auto.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1015,6 +1199,26 @@
           <t>GPIO firmware: A=4, B=19, SW=23.</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Encodeur THT, souvent manuel/wave</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1070,6 +1274,26 @@
           <t>Mettre sur PCB A. Pull-ups internes ESP32 insuffisants pour robustesse bus.</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>SMT Basic (si code LCSC valide)</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Pret cote reference LCSC (verifier stock JLC).</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1125,6 +1349,26 @@
           <t>Alternative: 2x B10B-XH-A (Mouser 455-B10B-XH-A, ~0.79/pc).</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>THT/Manual</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Completer un code LCSC (Cxxxx) pour PCBA auto.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1178,6 +1422,26 @@
       <c r="K13" s="2" t="inlineStr">
         <is>
           <t>Ajouter ESD + resistances serie 33-100R sur ports externes.</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>THT/Manual</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Completer un code LCSC (Cxxxx) pour PCBA auto.</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1203,10 +1467,14 @@
     <col width="6" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
     <col width="31" customWidth="1" min="7" max="7"/>
-    <col width="63" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
     <col width="5" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="67" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="35" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="52" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1265,6 +1533,26 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Assemble_JLC</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>JLC_Type</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>LCSC_Status</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>JLC_Notes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1320,6 +1608,26 @@
           <t>A appairer avec le header JST XH cote PCB A.</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Connectique cable/harness, pas composant SMT carte</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1375,6 +1683,26 @@
           <t>Le firmware est calibre pour 15k et B~3920.</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Sonde externe (off-board)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1430,6 +1758,26 @@
           <t>Firmware divisorValue=8400. Ajustable par calibration logicielle.</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>SMT Basic (si code LCSC valide)</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Completer un code LCSC (Cxxxx) pour PCBA auto.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1485,6 +1833,26 @@
           <t>Voir onglet MOSFET_3V3 pour comparaison detaillee.</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>THT (TO-220) ou SMT (AO3400A)</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Completer un code LCSC (Cxxxx) pour PCBA auto.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1540,6 +1908,26 @@
           <t>Rgate typ 100R; pull-down typ 100k.</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>SMT Basic (si code LCSC valide)</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Completer un code LCSC (Cxxxx) pour PCBA auto.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1595,6 +1983,26 @@
           <t>Dimensionner selon courant chauffage reel.</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Bornier THT, souvent manuel/wave</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1650,6 +2058,26 @@
           <t>Choisir tension TVS selon bus, fusible selon Imax.</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>SMT/THT selon choix</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Completer un code LCSC (Cxxxx) pour PCBA auto.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1705,6 +2133,26 @@
           <t>Limite bruit ADC et aliasing sur lecture temperature.</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>SMT Basic (si codes LCSC valides)</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Completer un code LCSC (Cxxxx) pour PCBA auto.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1760,6 +2208,26 @@
           <t>Peut stocker ID_B, calibration, revision.</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>SMT</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Completer un code LCSC (Cxxxx) pour PCBA auto.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1815,6 +2283,26 @@
           <t>Utile si precision mesure &gt; ADC ESP32 requise.</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>SMT</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Completer un code LCSC (Cxxxx) pour PCBA auto.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1868,6 +2356,26 @@
       <c r="K12" s="2" t="inlineStr">
         <is>
           <t>Permet remonter defaut vers PCB A (FAULT/INT).</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>SMT</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Completer un code LCSC (Cxxxx) pour PCBA auto.</t>
         </is>
       </c>
     </row>
@@ -1883,7 +2391,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -1897,7 +2405,8 @@
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="39" customWidth="1" min="10" max="10"/>
     <col width="40" customWidth="1" min="11" max="11"/>
-    <col width="70" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1961,6 +2470,11 @@
           <t>Usage conseille</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Recommended_for_this_project</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2023,6 +2537,11 @@
           <t>Prototype, PWM 500 Hz, courant modere</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Current baseline</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2085,6 +2604,11 @@
           <t>Remplacement direct de IRLZ44N en TO-220</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2147,6 +2671,11 @@
           <t>Courants eleves, bonne dissipation</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2207,6 +2736,11 @@
       <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Petites charges ou carte compacte</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
     </row>
@@ -2243,6 +2777,11 @@
       <c r="L7" s="3" t="inlineStr">
         <is>
           <t>Prendre un MOSFET avec Rds(on) spec a Vgs=2.5V/4.5V. Verifier P=I^2*Rds(on), temperature jonction, et marge thermique.</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Guideline</t>
         </is>
       </c>
     </row>
@@ -2361,7 +2900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2452,6 +2991,18 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PCBA JLC</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Utiliser Assemble_JLC=Yes comme scope; chaque ligne Yes doit avoir LCSC Cxxxx valide.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>